<commit_message>
Updated 9 files: app.py, crear_db.py, database.db, reporte.xlsx, requirements.txt, index.html, reporte_1777681610.png, 1777681610.png, 1777813117.png
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/reporte.xlsx
+++ b/reporte.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registros" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Registros" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46,8 +46,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -125,10 +128,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -140,20 +143,20 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>2</row>
       <rowOff>0</rowOff>
@@ -165,20 +168,20 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
@@ -190,20 +193,20 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>4</row>
       <rowOff>0</rowOff>
@@ -215,20 +218,20 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>5</row>
       <rowOff>0</rowOff>
@@ -240,20 +243,20 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
@@ -265,20 +268,20 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>5</col>
       <colOff>0</colOff>
       <row>7</row>
       <rowOff>0</rowOff>
@@ -290,13 +293,63 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="762000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -593,8 +646,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -614,168 +675,269 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Imagen</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="80" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>16:35:20.036237</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>12345678</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>sensor map</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="80" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>17:16:48.321673</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>12345678</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>tarjeta</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>17:24:31.821804</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>1515</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Pascal</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>luz en mal estado</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>17:25:11.832700</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>1717</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Pablo Escobar</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>plata o plomo</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>17:37:09.789956</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>1717</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Pablo Escobar</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>plata o plomo, tu decides marica</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>17:40:27.379405</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>1717</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Pablo Escobar</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>la luz se averio</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>17:43:28.774566</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>12345678</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Juan Perez</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>mal estado de la bomba</t>
         </is>
       </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>20:26:50.360299</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>1717</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Pablo Escobar</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>lsgb r gesrg es hset segs</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>08:58:37.447159</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>1515</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Pedro Pascal</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>los trabajadores estan trabajando sin casco</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="1" t="n"/>
+      <c r="C11" s="1" t="n"/>
+      <c r="D11" s="1" t="n"/>
+      <c r="E11" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>